<commit_message>
Cập nhật CS13 Đề 1 theo hồ sơ tình huống: 6 việc gợi ý, cổng theo quy tắc ba, giờ chuyên gia; thêm báo cáo nhóm và cá nhân
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFjaXE4k5JPrGpMNxZm1fr
</commit_message>
<xml_diff>
--- a/P100_CS13.xlsx
+++ b/P100_CS13.xlsx
@@ -774,7 +774,11 @@
           <t>Số liệu kinh tế của đề (9 dòng)</t>
         </is>
       </c>
-      <c r="B5" s="40" t="n"/>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C5" s="39" t="inlineStr">
         <is>
           <t>Đã điền sẵn ở trang 2, dòng 12–20: chi phí mỗi việc, biên lợi nhuận, điều kiện dừng</t>
@@ -785,7 +789,11 @@
           <t>Đọc để hiểu; không cần chép</t>
         </is>
       </c>
-      <c r="E5" s="40" t="n"/>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>254 + 200 đ/hóa đơn; duyệt 1,5 phút × 50.000 đ/giờ; doanh thu 3,97 triệu/1.760 hóa đơn = 2.256 đ/hóa đơn; hết tiền tháng 7</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="33.75" customHeight="1" s="33">
       <c r="A6" s="39" t="inlineStr">
@@ -793,7 +801,11 @@
           <t>Bối cảnh, sản phẩm, "1 việc" là gì</t>
         </is>
       </c>
-      <c r="B6" s="40" t="n"/>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
           <t>Giả thuyết và chỉ số ở trang 1</t>
@@ -806,7 +818,7 @@
       </c>
       <c r="E6" s="40" t="inlineStr">
         <is>
-          <t>"1 việc" = 1 hóa đơn được đọc và nhập; khách = văn phòng kế toán, bình quân 1.760 hóa đơn/tháng</t>
+          <t>1 việc = 1 hóa đơn được đọc, đối chiếu và nhập vào phần mềm kế toán. Văn phòng thử nghiệm: 40 doanh nghiệp, ~12.000 hóa đơn/tháng</t>
         </is>
       </c>
     </row>
@@ -816,7 +828,11 @@
           <t>6 việc gợi ý</t>
         </is>
       </c>
-      <c r="B7" s="40" t="n"/>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C7" s="39" t="inlineStr">
         <is>
           <t>Trang 1, cột B–C; nhóm được thêm việc của mình</t>
@@ -827,7 +843,11 @@
           <t>Giữ, bỏ hay đổi thứ tự đều phải ghi lý do ở cột Q</t>
         </is>
       </c>
-      <c r="E7" s="40" t="n"/>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>Đã chép đủ 6 việc vào trang 1; thêm việc 7 (kiểm chứng doanh thu bình quân)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="33">
       <c r="A8" s="39" t="inlineStr">
@@ -835,7 +855,11 @@
           <t>Kết quả đánh giá đã có (bộ đề, cổng phát hành)</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n"/>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Cổng đánh giá ở trang 2; việc cần làm trước ở trang 3</t>
@@ -846,7 +870,11 @@
           <t>Đề 2, 3: kết luận chưa phải "Phát hành" → có việc phải làm trước</t>
         </is>
       </c>
-      <c r="E8" s="40" t="n"/>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>Bản 2 PHÁT HÀNH: đạt 97,3% (ngưỡng 95%), 0 lỗi nghiêm trọng, 0 tầng tụt, kappa 0,90. Bộ đề 40 hóa đơn: Thường 65%, Khó 25%, Nguy hiểm 7%, Ngoài phạm vi 3%</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="33.75" customHeight="1" s="33">
       <c r="A9" s="39" t="inlineStr">
@@ -854,7 +882,11 @@
           <t>Chuyên gia và số giờ của họ</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n"/>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C9" s="39" t="inlineStr">
         <is>
           <t>Dòng "Điều kiện cần" ở trang 3; ô "Cần gì" ở trang 5</t>
@@ -867,7 +899,7 @@
       </c>
       <c r="E9" s="40" t="inlineStr">
         <is>
-          <t>Ghi đúng tên chuyên gia và số giờ theo hồ sơ (kế toán trưởng duyệt bộ đề)</t>
+          <t>Chị Hạnh (kế toán trưởng 15 năm) 3 giờ/tuần, sáng thứ Bảy; anh Tùng (trưởng nhóm nhập liệu 6 năm). 1 vòng chấm bộ đề 40 ca = 8,5 giờ</t>
         </is>
       </c>
     </row>
@@ -877,7 +909,11 @@
           <t>Gợi ý về người duyệt và mức tự động</t>
         </is>
       </c>
-      <c r="B10" s="40" t="n"/>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Trang 2, cột H và I</t>
@@ -888,7 +924,11 @@
           <t>Đề 3: bác sĩ của bệnh viện không tính vào chi phí</t>
         </is>
       </c>
-      <c r="E10" s="40" t="n"/>
+      <c r="E10" s="40" t="inlineStr">
+        <is>
+          <t>Người duyệt = kế toán viên của công ty. Mức 1 ~20% (gắn cờ + mẫu 10%), Mức 2 ~10%. 'Sai MST hay sai tiền thì không được lần nào'</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="33">
       <c r="A12" s="41" t="inlineStr">
@@ -1055,41 +1095,41 @@
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Đọc hóa đơn ảnh/PDF, tự trích trường (MST, số HĐ, ngày, tiền hàng, VAT)</t>
+          <t>Đọc ảnh hóa đơn giấy, ảnh chụp</t>
         </is>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>Giảm 50% giờ nhập hóa đơn ảnh của kế toán viên</t>
+          <t>Giảm 50% giờ nhập hóa đơn ảnh</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng làm đọc tự động hóa đơn ảnh/PDF cho kế toán viên văn phòng dịch vụ sẽ giảm 50% giờ nhập liệu, vì nhập tay là việc tốn giờ nhất mỗi tháng</t>
+          <t>Ta tin rằng dùng bản 2 đọc ảnh hóa đơn giấy cho kế toán viên của văn phòng dịch vụ sẽ giảm 50% giờ nhập hóa đơn ảnh mà không có lỗi MST hay số tiền</t>
         </is>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>Giờ nhập/100 hóa đơn giảm ≥ 50%; đúng ≥ 98% trường số tiền và MST trên 300 hóa đơn thật</t>
+          <t>Giờ nhập/100 hóa đơn ảnh giảm ≥ 50% so với nhập tay sau 30 ngày; 0 lỗi MST/tiền lọt vào sổ trên ≥ 3.000 hóa đơn ảnh</t>
         </is>
       </c>
       <c r="F5" s="40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G5" s="40" t="n">
         <v>5</v>
       </c>
       <c r="H5" s="40" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I5" s="40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" s="40" t="n">
         <v>0.8</v>
       </c>
       <c r="K5" s="40" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="L5" s="40" t="n">
         <v>0.4</v>
@@ -1113,7 +1153,7 @@
       </c>
       <c r="Q5" s="46" t="inlineStr">
         <is>
-          <t>Hạng 3 nhưng làm TRƯỚC: đây là lõi sản phẩm, đúng '1 việc' của đề (1 hóa đơn); việc hạng 1 và 2 chỉ có giá trị khi việc này chạy. Rủi ro bị nuốt 0,4: OCR chung khó với ảnh mờ, hóa đơn viết tay, mẫu Việt Nam</t>
+          <t>Hạng 4 nhưng làm ngay: bản 2 đã qua cổng phát hành (97,3%, 0 lỗi nghiêm trọng, kappa 0,90) nên mức tự tin 1, công sức thấp. Bị nuốt 0,4: OCR chung đọc được ảnh rõ nhưng khó với ảnh mờ, hóa đơn viết tay</t>
         </is>
       </c>
     </row>
@@ -1123,44 +1163,44 @@
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Đối chiếu hóa đơn với dữ liệu hóa đơn điện tử trên cổng thuế</t>
+          <t>Gắn cờ hóa đơn cần người xem</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>Phát hiện sai lệch trước khi kê khai</t>
+          <t>Kế toán chỉ xem khoảng 20% hóa đơn</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng đối chiếu tự động với hóa đơn điện tử cho kế toán viên sẽ giảm 70% lỗi kê khai do nhập sai</t>
+          <t>Ta tin rằng gắn cờ đúng các hóa đơn khó/nguy hiểm cho kế toán viên sẽ giúp họ chỉ phải xem ~20% hóa đơn mà vẫn không lọt lỗi MST hay tiền</t>
         </is>
       </c>
       <c r="E6" s="40" t="inlineStr">
         <is>
-          <t>Lỗi lệch số tiền/MST phát hiện sau kê khai giảm ≥ 70% trên 10 văn phòng thử</t>
+          <t>Tỷ lệ gắn cờ ≤ 20%, cờ thừa ≤ 10%; bắt 100% hóa đơn tầng Nguy hiểm trong bộ đề; 0 lỗi MST/tiền lọt qua trên ≥ 3.000 hóa đơn thật</t>
         </is>
       </c>
       <c r="F6" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="40" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I6" s="40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J6" s="40" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="K6" s="40" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="L6" s="40" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="M6" s="44">
         <f>IF(COUNT(F6:L6)&lt;7,"",ROUND(F6*G6*H6/I6*(0.5+0.5*AVERAGE(J6:K6))*(1-0.5*L6),2))</f>
@@ -1176,12 +1216,12 @@
       </c>
       <c r="P6" s="46" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>Tự làm</t>
         </is>
       </c>
       <c r="Q6" s="46" t="inlineStr">
         <is>
-          <t>Hạng 6. Chờ: cần quyền truy cập dữ liệu cổng thuế; phần mềm kế toán và nền tảng hóa đơn điện tử đã có tính năng tương tự (rủi ro bị nuốt 0,7). Xem lại ở ngày 90</t>
+          <t>Hạng 2, làm TRƯỚC cùng việc 4: đây là chìa khóa lên Mức 1 (duyệt 20%, biên 69%). Chị Hạnh: cờ thừa chấp nhận được nhưng không phải 1/2 số hóa đơn. Khó bị nuốt vì phải học theo luật và lỗi riêng của từng văn phòng</t>
         </is>
       </c>
     </row>
@@ -1191,44 +1231,44 @@
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Gợi ý định khoản (tài khoản nợ/có) cho từng hóa đơn</t>
+          <t>Nhập tự động hóa đơn điện tử (tệp gốc)</t>
         </is>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>Kế toán viên chỉ duyệt, không tự chọn tài khoản</t>
+          <t>Giảm 70% thời gian nhập hóa đơn điện tử</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng gợi ý định khoản dựa trên lịch sử của từng khách sẽ giúp kế toán viên giảm 30% thời gian hạch toán</t>
+          <t>Ta tin rằng nhập thẳng tệp gốc hóa đơn điện tử cho kế toán viên sẽ giảm 70% thời gian nhập loại hóa đơn này</t>
         </is>
       </c>
       <c r="E7" s="40" t="inlineStr">
         <is>
-          <t>Gợi ý được chấp nhận không sửa ≥ 80% trên 500 hóa đơn; thời gian hạch toán giảm ≥ 30%</t>
+          <t>Thời gian nhập/100 hóa đơn điện tử giảm ≥ 70%; ≥ 99% tệp gốc nhập không lỗi trên 1.000 hóa đơn</t>
         </is>
       </c>
       <c r="F7" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" s="40" t="n">
         <v>4</v>
       </c>
       <c r="H7" s="40" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I7" s="40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" s="40" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="K7" s="40" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L7" s="40" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="M7" s="44">
         <f>IF(COUNT(F7:L7)&lt;7,"",ROUND(F7*G7*H7/I7*(0.5+0.5*AVERAGE(J7:K7))*(1-0.5*L7),2))</f>
@@ -1244,12 +1284,12 @@
       </c>
       <c r="P7" s="46" t="inlineStr">
         <is>
-          <t>Tự làm</t>
+          <t>Mua</t>
         </is>
       </c>
       <c r="Q7" s="46" t="inlineStr">
         <is>
-          <t>Hạng 5, để tầng Tiếp theo: cần Mức 1 ổn định và đủ lịch sử định khoản của từng khách</t>
+          <t>Hạng 5. Mua (dùng sẵn): phần mềm kế toán văn phòng đang dùng ĐÃ CÓ tính năng nhập hóa đơn điện tử từ tệp gốc → rủi ro bị nuốt 1. Chỉ nối luồng: hóa đơn điện tử đi qua đối chiếu MST + gắn cờ của mình rồi nhập bằng tính năng sẵn có</t>
         </is>
       </c>
     </row>
@@ -1259,44 +1299,44 @@
       </c>
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Phát hiện hóa đơn trùng, MST ngừng hoạt động, sai thuế suất</t>
+          <t>Đối chiếu mã số thuế người bán</t>
         </is>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>Chặn hóa đơn rủi ro trước khi nhập sổ</t>
+          <t>Không nhập nhầm người bán</t>
         </is>
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng cảnh báo hóa đơn trùng/sai cho kế toán viên sẽ giúp phát hiện ≥ 90% hóa đơn lỗi trước khi nhập sổ</t>
+          <t>Ta tin rằng tự đối chiếu MST người bán với dịch vụ tra cứu cho mọi hóa đơn sẽ giúp kế toán viên không nhập nhầm người bán lần nào</t>
         </is>
       </c>
       <c r="E8" s="40" t="inlineStr">
         <is>
-          <t>Bắt được ≥ 90% hóa đơn lỗi cài sẵn trong 200 ca; báo nhầm &lt; 5%</t>
+          <t>0 hóa đơn nhầm/sai MST người bán lọt vào sổ trên ≥ 3.000 hóa đơn thật (quy tắc ba: lỗi thật &lt; 0,1%); 100% MST sai/ngừng hoạt động bị gắn cờ</t>
         </is>
       </c>
       <c r="F8" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" s="40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H8" s="40" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I8" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="40" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L8" s="40" t="n">
         <v>0.7</v>
-      </c>
-      <c r="K8" s="40" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="L8" s="40" t="n">
-        <v>0.5</v>
       </c>
       <c r="M8" s="44">
         <f>IF(COUNT(F8:L8)&lt;7,"",ROUND(F8*G8*H8/I8*(0.5+0.5*AVERAGE(J8:K8))*(1-0.5*L8),2))</f>
@@ -1312,12 +1352,12 @@
       </c>
       <c r="P8" s="46" t="inlineStr">
         <is>
-          <t>Tự làm</t>
+          <t>Mua</t>
         </is>
       </c>
       <c r="Q8" s="46" t="inlineStr">
         <is>
-          <t>Hạng 4: công sức thấp, dùng luật đơn giản trên dữ liệu đã trích ở việc 1; đi kèm việc 1 làm lớp kiểm tra an toàn</t>
+          <t>Hạng 1. Mua: tích hợp dịch vụ tra cứu MST có sẵn, không tự xây. Làm TRƯỚC vì 'sai MST thì không được lần nào' (chị Hạnh) và công sức thấp nhất</t>
         </is>
       </c>
     </row>
@@ -1327,44 +1367,44 @@
       </c>
       <c r="B9" s="40" t="inlineStr">
         <is>
-          <t>Xuất file nhập thẳng vào phần mềm kế toán đang dùng</t>
+          <t>Gợi ý tài khoản hạch toán</t>
         </is>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>Không phải gõ lại sau khi AI đọc</t>
+          <t>Giảm 30% thời gian hạch toán</t>
         </is>
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng xuất đúng định dạng nhập của phần mềm kế toán cho văn phòng sẽ giúp ≥ 90% hóa đơn đã đọc vào sổ không cần gõ lại</t>
+          <t>Ta tin rằng gợi ý tài khoản hạch toán theo lịch sử của từng doanh nghiệp cho kế toán viên sẽ giảm 30% thời gian hạch toán</t>
         </is>
       </c>
       <c r="E9" s="40" t="inlineStr">
         <is>
-          <t>≥ 90% hóa đơn nhập thành công không lỗi định dạng trên 10 văn phòng thử</t>
+          <t>Thời gian hạch toán/100 hóa đơn giảm ≥ 30%; ≥ 80% gợi ý được chấp nhận không sửa trên 500 hóa đơn</t>
         </is>
       </c>
       <c r="F9" s="40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9" s="40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H9" s="40" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9" s="40" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="K9" s="40" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="L9" s="40" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="M9" s="44">
         <f>IF(COUNT(F9:L9)&lt;7,"",ROUND(F9*G9*H9/I9*(0.5+0.5*AVERAGE(J9:K9))*(1-0.5*L9),2))</f>
@@ -1380,12 +1420,12 @@
       </c>
       <c r="P9" s="46" t="inlineStr">
         <is>
-          <t>Tự làm</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="Q9" s="46" t="inlineStr">
         <is>
-          <t>Hạng 2: công sức thấp, tự tin cao; làm cùng việc 1 vì không có file nhập vào sổ thì không giảm được giờ nhập</t>
+          <t>Hạng 6. Chờ: CHƯA có dữ liệu hạch toán của doanh nghiệp khách hàng (sẵn sàng dữ liệu 0,1) và chưa có bộ đề. Bắt đầu thu dữ liệu hạch toán từ tháng 1; xem lại ở ngày 90</t>
         </is>
       </c>
     </row>
@@ -1395,26 +1435,26 @@
       </c>
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Trợ lý hỏi đáp thuế, kế toán chung</t>
+          <t>Trả lời câu hỏi thuế chung cho khách của văn phòng</t>
         </is>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>Kế toán viên tra cứu nhanh</t>
+          <t>Bớt cuộc gọi hỏi đáp</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng trợ lý trả lời câu hỏi thuế chung sẽ giúp kế toán viên tiết kiệm thời gian tra cứu</t>
+          <t>Ta tin rằng trả lời câu hỏi thuế chung cho khách của văn phòng sẽ giảm cuộc gọi hỏi đáp</t>
         </is>
       </c>
       <c r="E10" s="40" t="inlineStr">
         <is>
-          <t>Điểm hài lòng ≥ 4/5 trên 100 câu hỏi</t>
+          <t>Số cuộc gọi hỏi đáp/tháng giảm ≥ 30%; ≥ 95% câu trả lời đúng trên 100 câu do chị Hạnh chấm</t>
         </is>
       </c>
       <c r="F10" s="40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" s="40" t="n">
         <v>2</v>
@@ -1426,10 +1466,10 @@
         <v>3</v>
       </c>
       <c r="J10" s="40" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K10" s="40" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L10" s="40" t="n">
         <v>0.9</v>
@@ -1453,7 +1493,7 @@
       </c>
       <c r="Q10" s="46" t="inlineStr">
         <is>
-          <t>Hạng 7. Không làm: mô hình miễn phí đã làm được (rủi ro bị nuốt 0,9), trả lời sai về thuế gây hại, không gắn với '1 việc' là hóa đơn</t>
+          <t>Hạng 7. Không làm: mô hình miễn phí đã trả lời được (bị nuốt 0,9); trả lời sai về thuế gây rủi ro cho văn phòng; ngoài '1 việc' là hóa đơn; tốn giờ chuyên gia vốn chỉ 3 giờ/tuần</t>
         </is>
       </c>
     </row>
@@ -1463,22 +1503,22 @@
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>Kiểm chứng gói giá với 30% văn phòng dùng nhiều</t>
+          <t>Kiểm chứng doanh thu với 30% văn phòng dùng nhiều</t>
         </is>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
-          <t>Biết văn phòng dùng nhiều có giữ mức trả hiện tại không</t>
+          <t>Biết doanh thu bình quân có giữ ≥ 3,71 triệu/văn phòng</t>
         </is>
       </c>
       <c r="D11" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng văn phòng dùng nhiều (65% doanh thu) vẫn trả đủ khi tính theo số hóa đơn, giữ doanh thu bình quân ≥ 3,71 triệu/văn phòng</t>
+          <t>Ta tin rằng 30% văn phòng dùng nhiều (65% doanh thu) sẽ gia hạn ở giá hiện tại khi SổSạch giảm được giờ nhập, giữ doanh thu bình quân ≥ 3,71 triệu/văn phòng</t>
         </is>
       </c>
       <c r="E11" s="40" t="inlineStr">
         <is>
-          <t>Doanh thu bình quân ≥ 3,71 triệu/văn phòng/tháng trên ≥ 10 văn phòng; ≥ 70% văn phòng dùng nhiều gia hạn</t>
+          <t>Doanh thu bình quân ≥ 3,71 triệu/văn phòng/tháng trên ≥ 10 văn phòng, 2 tháng liên tiếp; ≥ 80% văn phòng dùng nhiều gia hạn</t>
         </is>
       </c>
       <c r="F11" s="40" t="n">
@@ -1494,13 +1534,13 @@
         <v>1</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K11" s="40" t="n">
         <v>0.8</v>
       </c>
       <c r="L11" s="40" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="44">
         <f>IF(COUNT(F11:L11)&lt;7,"",ROUND(F11*G11*H11/I11*(0.5+0.5*AVERAGE(J11:K11))*(1-0.5*L11),2))</f>
@@ -1521,7 +1561,7 @@
       </c>
       <c r="Q11" s="46" t="inlineStr">
         <is>
-          <t>Hạng 1. Thêm việc: kiểm chứng biến nguy hiểm nhất của đề (65% doanh thu từ 30% văn phòng dùng nhiều). Không cần xây thêm tính năng</t>
+          <t>Hạng 3. Thêm việc: kiểm chứng biến nguy hiểm nhất của đề (doanh thu bình quân). Không cần xây tính năng; cần để quyết định ở ngày 90 trước khi hết tiền tháng 7</t>
         </is>
       </c>
     </row>
@@ -1756,27 +1796,27 @@
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>AI đọc hóa đơn, điền sẵn các trường</t>
+          <t>AI đọc hóa đơn (ảnh + tệp gốc), tra MST, điền sẵn và gắn cờ</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Kế toán viên của công ty đối chiếu 100% với ảnh gốc, sửa rồi gửi</t>
+          <t>Kế toán viên của công ty xem 100% hóa đơn, đối chiếu ảnh gốc, sửa rồi nhập; chị Hạnh kiểm 1% hóa đơn thật, đếm riêng cờ thừa</t>
         </is>
       </c>
       <c r="E5" s="40" t="inlineStr">
         <is>
-          <t>— (mức khởi đầu)</t>
+          <t>— (mức khởi đầu; bản 2 đã qua cổng phát hành: 97,3%, 0 lỗi nghiêm trọng, kappa 0,90)</t>
         </is>
       </c>
       <c r="F5" s="40" t="inlineStr">
         <is>
-          <t>Thu ảnh/PDF hóa đơn; lưu ảnh gốc để tra lại; báo khách biết dữ liệu do AI đọc (Luật AI 134/2025/QH15); thỏa thuận xử lý dữ liệu với văn phòng</t>
+          <t>Tích hợp dịch vụ tra cứu MST; lưu ảnh/tệp gốc để tra lại; nhật ký sửa; thông báo cho văn phòng biết dữ liệu do AI đọc (Luật AI 134/2025/QH15, NĐ 142/2026 Điều 18); thỏa thuận xử lý dữ liệu</t>
         </is>
       </c>
       <c r="G5" s="40" t="inlineStr">
         <is>
-          <t>T1–T2</t>
+          <t>Tháng 1</t>
         </is>
       </c>
       <c r="H5" s="47" t="n">
@@ -1811,27 +1851,27 @@
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>AI tự nhập hóa đơn rõ, độ tin cậy cao; hóa đơn khó vào hàng chờ duyệt</t>
+          <t>AI tự nhập hóa đơn không gắn cờ; hóa đơn gắn cờ vào hàng chờ</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Duyệt mẫu ngẫu nhiên + mọi hóa đơn AI không chắc (khoảng 20%)</t>
+          <t>Kế toán viên duyệt mọi hóa đơn gắn cờ + mẫu ngẫu nhiên 10% (~20%); chị Hạnh kiểm 1%</t>
         </is>
       </c>
       <c r="E6" s="40" t="inlineStr">
         <is>
-          <t>Đúng ≥ 98% trường số tiền và MST trên ≥ 300 hóa đơn thật (bộ đề có nhãn); sai số tiền &gt; 1% = 0 ca; kế toán trưởng xác nhận</t>
+          <t>0 lỗi MST/tiền trên ≥ 3.000 hóa đơn thật đã duyệt 100% ở Mức 0 (quy tắc ba: lỗi thật &lt; 0,1%); gắn cờ ≤ 20%, cờ thừa ≤ 10%; bộ đề 40 ca không tầng tụt; chị Hạnh xác nhận</t>
         </is>
       </c>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>Bộ đề 300 hóa đơn có nhãn (đủ ảnh mờ, viết tay, nhiều trang); nhật ký sửa; bảng giám sát độ chính xác theo trường</t>
+          <t>Hàng chờ duyệt theo cờ; bảng giám sát lỗi MST/tiền, tỷ lệ cờ; cảnh báo ngay khi có 1 lỗi MST/tiền</t>
         </is>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
-          <t>T3–T4</t>
+          <t>Tháng 2–3</t>
         </is>
       </c>
       <c r="H6" s="47" t="n">
@@ -1870,27 +1910,27 @@
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>AI tự nhập và xuất file vào phần mềm kế toán; tự chuyển người khi độ tin cậy thấp</t>
+          <t>AI tự nhập và tự chuyển hóa đơn độ tin cậy thấp cho người; xử lý ≥ 3 văn phòng</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Xử lý ca chuyển lên; kiểm tra ngẫu nhiên khoảng 10%</t>
+          <t>Duyệt hóa đơn gắn cờ + mẫu 5% (~10%); anh Tùng chấm lại bộ đề mỗi lần đổi mô hình</t>
         </is>
       </c>
       <c r="E7" s="40" t="inlineStr">
         <is>
-          <t>Tỷ lệ sửa của người duyệt &lt; 5% trên ≥ 1.000 hóa đơn thực tế của ≥ 10 văn phòng; bắt ≥ 90% hóa đơn lỗi cài sẵn; khiếu nại &lt; 1%; kế toán trưởng + quản lý sản phẩm xác nhận</t>
+          <t>0 lỗi MST/tiền trên ≥ 10.000 hóa đơn thật của ≥ 3 văn phòng (lỗi thật &lt; 0,03%); cờ thừa ≤ 5%; bộ đề mở rộng ≥ 80 ca, tỷ lệ đạt quy về thực tế ≥ 97%; chị Hạnh + quản lý sản phẩm xác nhận</t>
         </is>
       </c>
       <c r="F7" s="40" t="inlineStr">
         <is>
-          <t>Mở rộng bộ đề 1.000 hóa đơn; tích hợp xuất file phần mềm kế toán; quy trình xử lý khiếu nại</t>
+          <t>Mở rộng bộ đề lên ≥ 80 ca (thêm tầng Nguy hiểm); quy trình khiếu nại; anh Tùng chấm chính để tiết kiệm giờ chị Hạnh</t>
         </is>
       </c>
       <c r="G7" s="40" t="inlineStr">
         <is>
-          <t>T5–T7</t>
+          <t>Tháng 4–6 (nếu qua cổng)</t>
         </is>
       </c>
       <c r="H7" s="47" t="n">
@@ -1929,27 +1969,27 @@
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>AI tự nhập, đối chiếu và gợi ý định khoản</t>
+          <t>AI tự nhập gần hết; chỉ hóa đơn Nguy hiểm/Ngoài phạm vi chuyển người</t>
         </is>
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Theo dõi bảng giám sát; kiểm tra mẫu 5% và ngoại lệ</t>
+          <t>Theo dõi bảng giám sát; kiểm mẫu 5% và ngoại lệ</t>
         </is>
       </c>
       <c r="E8" s="40" t="inlineStr">
         <is>
-          <t>Lỗi phát hiện sau kê khai ≤ 0,5% trên ≥ 3.000 hóa đơn trong 2 tháng liên tục; không có lỗi số tiền lớn; ban lãnh đạo duyệt</t>
+          <t>0 lỗi MST/tiền trên ≥ 30.000 hóa đơn thật trong 2 tháng trên ≥ 10 văn phòng (lỗi thật &lt; 0,01%); khiếu nại &lt; 0,5%; ban lãnh đạo duyệt</t>
         </is>
       </c>
       <c r="F8" s="40" t="inlineStr">
         <is>
-          <t>Truy cập dữ liệu hóa đơn điện tử; lưu vết đầy đủ; rà soát mức rủi ro theo Luật AI</t>
+          <t>Lưu vết đầy đủ để tra lại khi quyết toán; rà soát mức rủi ro theo Luật AI</t>
         </is>
       </c>
       <c r="G8" s="40" t="inlineStr">
         <is>
-          <t>T8+</t>
+          <t>Chưa hứa ngày: chỉ khi qua cổng</t>
         </is>
       </c>
       <c r="H8" s="47" t="n">
@@ -2208,17 +2248,17 @@
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Đọc hóa đơn ảnh/PDF (việc 1) + xuất file vào phần mềm kế toán (việc 5) + cảnh báo hóa đơn lỗi (việc 4) + kiểm chứng gói giá với văn phòng dùng nhiều (việc 7)</t>
+          <t>Đối chiếu MST người bán (hạng 1, Mua: tích hợp dịch vụ tra cứu) + gắn cờ hóa đơn cần người xem (hạng 2) + vận hành bản 2 đọc ảnh (hạng 4) + kiểm chứng doanh thu văn phòng dùng nhiều (hạng 3)</t>
         </is>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>Tự động một phần (Mức 2) + gợi ý định khoản (việc 3)</t>
+          <t>Mức 2 cho ≥ 3 văn phòng; bắt đầu thu dữ liệu hạch toán cho việc 5</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Đối chiếu với hóa đơn điện tử (việc 2, nếu chưa bị nuốt); thử Mức 3</t>
+          <t>Gợi ý tài khoản hạch toán (việc 5) nếu đủ dữ liệu; xem xét Mức 3</t>
         </is>
       </c>
     </row>
@@ -2230,17 +2270,17 @@
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Ta tin rằng đọc tự động hóa đơn ảnh cho kế toán viên sẽ giảm 50% giờ nhập liệu, và văn phòng dùng nhiều vẫn trả đủ để doanh thu bình quân ≥ 3,71 triệu</t>
+          <t>Ta tin rằng đối chiếu MST + gắn cờ đúng cho kế toán viên sẽ giúp họ chỉ xem ~20% hóa đơn, giảm 50% giờ nhập hóa đơn ảnh, không lọt lỗi MST/tiền; văn phòng dùng nhiều sẽ gia hạn</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>Có người duyệt ở Mức 1 → văn phòng tin dùng → giảm duyệt còn 10%</t>
+          <t>Gắn cờ ổn định → giảm duyệt còn 10% mà vẫn 0 lỗi MST/tiền</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Đối chiếu tự động giảm lỗi kê khai</t>
+          <t>Đủ lịch sử hạch toán → gợi ý giảm 30% thời gian hạch toán</t>
         </is>
       </c>
     </row>
@@ -2252,17 +2292,17 @@
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Giờ nhập/100 hóa đơn giảm ≥ 50%; đúng ≥ 98% trường số tiền, MST; doanh thu bình quân ≥ 3,71 triệu/văn phòng</t>
+          <t>0 lỗi MST/tiền lọt vào sổ; gắn cờ ≤ 20%, cờ thừa ≤ 10%; giờ nhập hóa đơn ảnh giảm ≥ 50%; doanh thu bình quân ≥ 3,71 triệu/văn phòng</t>
         </is>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>Tỷ lệ sửa &lt; 5%; gợi ý định khoản được chấp nhận ≥ 80%</t>
+          <t>Cờ thừa ≤ 5%; 0 lỗi MST/tiền trên ≥ 10.000 hóa đơn</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>Lỗi phát hiện sau kê khai giảm ≥ 70%</t>
+          <t>≥ 80% gợi ý được chấp nhận không sửa</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2314,7 @@
       </c>
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Mức 0 → Mức 1 (duyệt 20%)</t>
+          <t>Mức 0 (duyệt 100%) tháng 1 → Mức 1 (duyệt 20%) tháng 2–3</t>
         </is>
       </c>
       <c r="C8" s="40" t="inlineStr">
@@ -2284,7 +2324,7 @@
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Thử Mức 3 (duyệt 5%)</t>
+          <t>Thử Mức 3 (duyệt 5%), không hứa ngày</t>
         </is>
       </c>
     </row>
@@ -2296,17 +2336,17 @@
       </c>
       <c r="B9" s="40" t="inlineStr">
         <is>
-          <t>Lên Mức 1: đúng ≥ 98% số tiền và MST trên ≥ 300 hóa đơn thật; 0 ca sai số tiền &gt; 1%; kế toán trưởng xác nhận</t>
+          <t>Lên Mức 1: 0 lỗi MST/tiền trên ≥ 3.000 hóa đơn thật (lỗi thật &lt; 0,1%); gắn cờ ≤ 20%, cờ thừa ≤ 10%; bộ đề 40 ca không tầng tụt; chị Hạnh xác nhận</t>
         </is>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>Sửa &lt; 5% trên ≥ 1.000 hóa đơn của ≥ 10 văn phòng; khiếu nại &lt; 1%</t>
+          <t>0 lỗi MST/tiền trên ≥ 10.000 hóa đơn của ≥ 3 văn phòng; bộ đề ≥ 80 ca đạt ≥ 97%</t>
         </is>
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>Lỗi sau kê khai ≤ 0,5% trên ≥ 3.000 hóa đơn trong 2 tháng</t>
+          <t>0 lỗi MST/tiền trên ≥ 30.000 hóa đơn trong 2 tháng, ≥ 10 văn phòng</t>
         </is>
       </c>
     </row>
@@ -2318,17 +2358,17 @@
       </c>
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Bộ đề 300 hóa đơn có nhãn (ảnh mờ, viết tay, nhiều trang); lưu ảnh gốc; báo khách dữ liệu do AI đọc theo Luật AI 134/2025/QH15; thỏa thuận xử lý dữ liệu; giờ kế toán trưởng gắn nhãn theo hồ sơ</t>
+          <t>Tích hợp dịch vụ tra cứu MST; lưu ảnh/tệp gốc; nhật ký sửa; thông báo dữ liệu do AI đọc (Luật AI, NĐ 142/2026 Điều 18); chị Hạnh 3 giờ/tuần kiểm 1% (~120 hóa đơn/tháng ≈ 3 giờ), anh Tùng chấm bộ đề (8,5 giờ/vòng)</t>
         </is>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>Bộ đề 1.000 hóa đơn; lịch sử định khoản từng khách; tích hợp phần mềm kế toán</t>
+          <t>Bộ đề ≥ 80 ca; quy trình khiếu nại; dữ liệu hạch toán có đồng ý của doanh nghiệp</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>Quyền truy cập dữ liệu hóa đơn điện tử; lưu vết; rà soát Luật AI</t>
+          <t>Dữ liệu hạch toán đủ 6 tháng; lưu vết khi quyết toán; rà soát Luật AI</t>
         </is>
       </c>
     </row>
@@ -2340,12 +2380,12 @@
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>Doanh thu 2.256 đ/hóa đơn (3,97 triệu ÷ 1.760). Mức 0 chi phí 1.704 đ → biên 24%; Mức 1 chi phí 704 đ → biên 69%. Kịch bản xấu hết tiền tháng 7 → rút ngắn Mức 0, thử 10–15 văn phòng</t>
+          <t>Doanh thu 2.256 đ/hóa đơn (3,97 triệu ÷ 1.760). Mức 0: 1.704 đ → biên 24%; Mức 1: 704 đ → biên 69%. Kịch bản xấu hết tiền tháng 7 → phải lên Mức 1 trong 3 tháng đầu</t>
         </is>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
-          <t>Mức 2 chi phí 579 đ → biên 74%; mở rộng khi doanh thu bình quân ≥ 3,71 triệu</t>
+          <t>Mức 2: 579 đ → biên 74%; mở rộng chỉ khi doanh thu bình quân ≥ 3,71 triệu</t>
         </is>
       </c>
       <c r="D11" s="40" t="inlineStr">
@@ -2362,17 +2402,17 @@
       </c>
       <c r="B12" s="40" t="inlineStr">
         <is>
-          <t>Nếu doanh thu bình quân &lt; 3,71 triệu/văn phòng trong 2 tháng liên tiếp trên ≥ 10 văn phòng, hoặc giờ nhập giảm &lt; 30% ở ngày 60 → dừng mở rộng, thiết kế lại gói giá</t>
+          <t>NẾU 1 lỗi MST/tiền lọt vào sổ THÌ lùi ngay về Mức 0. NẾU ngày 60 tỷ lệ gắn cờ &gt; 35% THÌ giữ Mức 0, sửa luật gắn cờ. NẾU doanh thu bình quân &lt; 3,71 triệu/văn phòng 2 tháng liên tiếp trên ≥ 10 văn phòng THÌ dừng mở rộng</t>
         </is>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
-          <t>Khiếu nại &gt; 2% hoặc sai số tiền tăng → lùi về Mức 1</t>
+          <t>Có lỗi MST/tiền hoặc khiếu nại &gt; 1% → lùi về Mức 1</t>
         </is>
       </c>
       <c r="D12" s="40" t="inlineStr">
         <is>
-          <t>Phần mềm kế toán/cổng thuế ra tính năng đọc hóa đơn miễn phí → bỏ đọc chung, tập trung hóa đơn khó và định khoản</t>
+          <t>Phần mềm kế toán ra tính năng đọc ảnh/gắn cờ tương tự miễn phí → bỏ việc bị nuốt, tập trung gợi ý hạch toán</t>
         </is>
       </c>
     </row>
@@ -2442,17 +2482,17 @@
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Giờ nhập/100 hóa đơn; tỷ lệ trường AI đọc đúng; số văn phòng đang dùng</t>
+          <t>Số lỗi MST/tiền (phải = 0); tỷ lệ gắn cờ và cờ thừa (chị Hạnh kiểm 1%); giờ nhập/100 hóa đơn ảnh</t>
         </is>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>Đi tiếp / Sửa (cách chụp ảnh, mẫu hóa đơn khó)</t>
+          <t>Đi tiếp / Sửa (luật gắn cờ, cách chụp ảnh)</t>
         </is>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
-          <t>Quản lý sản phẩm + kế toán trưởng</t>
+          <t>Quản lý sản phẩm + chị Hạnh</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2504,7 @@
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Cổng Mức 0 → 1: đúng ≥ 98% số tiền, MST trên 300 hóa đơn; giờ nhập giảm ≥ 30%; chi phí mỗi hóa đơn thực tế</t>
+          <t>Cổng Mức 0 → 1: 0 lỗi MST/tiền trên ≥ 3.000 hóa đơn; gắn cờ ≤ 20%, cờ thừa ≤ 10%; chi phí mỗi hóa đơn thực tế</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
@@ -2474,7 +2514,7 @@
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Quản lý sản phẩm + trưởng nhóm kỹ thuật + kế toán trưởng</t>
+          <t>Quản lý sản phẩm + trưởng nhóm kỹ thuật + chị Hạnh</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2526,12 @@
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Doanh thu bình quân so với 3,71 triệu (2 tháng, ≥ 10 văn phòng); giờ nhập giảm ≥ 50%; tỷ lệ văn phòng dùng nhiều gia hạn</t>
+          <t>Doanh thu bình quân so với 3,71 triệu (2 tháng, ≥ 10 văn phòng); tỷ lệ văn phòng dùng nhiều gia hạn; biên ở Mức 1 ≥ 60%</t>
         </is>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>Đi tiếp (mở rộng) / Đổi hướng (gói giá) / Dừng</t>
+          <t>Đi tiếp (mở rộng) / Đổi hướng (gói giá) / Dừng mở rộng; quyết định có làm việc 5</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
@@ -2508,12 +2548,12 @@
       </c>
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Chạy lại bộ đề 300 hóa đơn; tính lại chi phí gọi AI (hiện 254 đ/hóa đơn)</t>
+          <t>Anh Tùng chạy lại bộ đề 40 ca (8,5 giờ) trên mô hình mới; tính lại chi phí gọi AI (hiện 254 đ/hóa đơn)</t>
         </is>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>Đổi mô hình? Hạ giá? Lên Mức 2 sớm hơn?</t>
+          <t>Đổi mô hình? Hạ giá? Giữ nguyên mức tự động cho đến khi qua cổng lại</t>
         </is>
       </c>
       <c r="D8" s="40" t="inlineStr">
@@ -2530,12 +2570,12 @@
       </c>
       <c r="B9" s="40" t="inlineStr">
         <is>
-          <t>Việc nào bị 'nuốt' (đọc hóa đơn, đối chiếu cổng thuế)</t>
+          <t>Phần mềm kế toán hoặc dịch vụ tra cứu MST ra tính năng đọc ảnh/gắn cờ</t>
         </is>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>Bỏ việc bị nuốt, dồn lực vào hóa đơn khó và định khoản</t>
+          <t>Bỏ việc bị nuốt, dồn lực vào gắn cờ theo từng văn phòng và gợi ý hạch toán</t>
         </is>
       </c>
       <c r="D9" s="40" t="inlineStr">
@@ -2552,12 +2592,12 @@
       </c>
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Mức rủi ro theo Luật AI 134/2025/QH15; quy định hóa đơn điện tử, bảo vệ dữ liệu cá nhân</t>
+          <t>Mức rủi ro theo Luật AI 134/2025/QH15; NĐ 142/2026 (thông báo, gắn nhãn); hạn chuyển tiếp Điều 35</t>
         </is>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>Thêm kiểm soát, nghĩa vụ thông báo, lưu vết</t>
+          <t>Thêm kiểm soát, thông báo, lưu vết; cập nhật cổng</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
@@ -2630,7 +2670,7 @@
       </c>
       <c r="B4" s="40" t="inlineStr">
         <is>
-          <t>Thử 3 tháng với 10–15 văn phòng: AI đọc hóa đơn ảnh giảm ≥ 50% giờ nhập, đúng ≥ 98% số tiền; ngày 90 quyết định mở rộng theo doanh thu ≥ 3,71 triệu/văn phòng.</t>
+          <t>Lên Mức 1 trong 3 tháng: kế toán chỉ xem 20% hóa đơn, 0 lỗi MST/tiền trên 3.000 hóa đơn, biên 69%; ngày 90 quyết định mở rộng nếu doanh thu ≥ 3,71 triệu/văn phòng.</t>
         </is>
       </c>
       <c r="C4" s="58">
@@ -2650,7 +2690,7 @@
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Bây giờ: đọc hóa đơn + xuất file phần mềm kế toán + cảnh báo lỗi + kiểm chứng gói giá · Tiếp theo: Mức 2, gợi ý định khoản · Sau này: đối chiếu hóa đơn điện tử</t>
+          <t>Bây giờ: đối chiếu MST + gắn cờ + đọc ảnh bản 2 + kiểm chứng doanh thu · Tiếp theo: Mức 2 (duyệt 10%), thu dữ liệu hạch toán · Sau này: gợi ý hạch toán</t>
         </is>
       </c>
       <c r="C5" s="58">
@@ -2670,7 +2710,7 @@
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>Kế toán viên duyệt 100% rồi 20%; giờ kế toán trưởng gắn nhãn 300 hóa đơn; ảnh hóa đơn thật của 10–15 văn phòng; thỏa thuận xử lý dữ liệu</t>
+          <t>Chị Hạnh 3 giờ/tuần kiểm 1% hóa đơn; anh Tùng chấm bộ đề (8,5 giờ/vòng); tích hợp dịch vụ tra cứu MST; ≥ 10 văn phòng thử nghiệm</t>
         </is>
       </c>
       <c r="C6" s="58">
@@ -2690,7 +2730,7 @@
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Doanh thu phụ thuộc 30% văn phòng dùng nhiều (65%) → kiểm chứng gói giá ngay; Mức 0 biên 24% → lên Mức 1 (biên 69%) sớm khi qua cổng</t>
+          <t>Doanh thu phụ thuộc 30% văn phòng dùng nhiều (65%), hết tiền tháng 7 → kiểm chứng gia hạn ngay; 1 lỗi MST/tiền → lùi Mức 0</t>
         </is>
       </c>
       <c r="C7" s="58">
@@ -2710,7 +2750,7 @@
       </c>
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Ngày 30/60/90; khi có mô hình mới, phần mềm kế toán ra tính năng tương tự hoặc Luật AI đổi</t>
+          <t>Ngày 30/60/90; khi có mô hình mới, phần mềm kế toán ra tính năng tương tự hoặc quy định AI thay đổi</t>
         </is>
       </c>
       <c r="C8" s="58">

</xml_diff>